<commit_message>
Clear a stray Professor title from two clinical team members
Yujin Lee and Sungeun Hong picked up the title by mistake when the
People sheet was reordered: the rows moved, but two old cells were not
cleared.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/glory-content.xlsx
+++ b/content/glory-content.xlsx
@@ -1464,11 +1464,7 @@
         </is>
       </c>
       <c r="B24" s="4" t="n"/>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Professor</t>
-        </is>
-      </c>
+      <c r="C24" s="4" t="n"/>
       <c r="D24" s="4" t="inlineStr">
         <is>
           <t>Clinical Research Team</t>
@@ -1491,11 +1487,7 @@
         </is>
       </c>
       <c r="B25" s="4" t="n"/>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Professor</t>
-        </is>
-      </c>
+      <c r="C25" s="4" t="n"/>
       <c r="D25" s="4" t="inlineStr">
         <is>
           <t>Clinical Research Team</t>

</xml_diff>

<commit_message>
Add the pizza party photo with screens covered; add professor emails
Gallery: 2026-10 pizzaparty now holds a version of the photo in which
the projector screen, its reflection in the glass wall, the laptop
screen in the foreground and a printed sheet are blurred.

People: add email addresses for the four principal investigators.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content/glory-content.xlsx
+++ b/content/glory-content.xlsx
@@ -815,7 +815,11 @@
           <t>Principal Investigators</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>jungyunlee@yuhs.ac</t>
+        </is>
+      </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>https://sev.severance.healthcare/sev/doctor/doctor-view.do?empNo=eXVoczIwMjBAKUApNMQSi3kCFf9SVaDJDBFLMqixdc0Mib9fT%2F4IUaKVBiU%3D&amp;deptSeq=87</t>
@@ -890,7 +894,11 @@
           <t>Principal Investigators</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n"/>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>svass@yuhs.ac</t>
+        </is>
+      </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>https://sev.severance.healthcare/sev/doctor/doctor-view.do?empNo=eXVoczIwMjBAKUApNMQSi0M%2BFf1aVaDJDRlLN%2FyizqbvK7rXBJaboa7jN3U%3D&amp;deptSeq=87</t>
@@ -961,7 +969,11 @@
           <t>Principal Investigators</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n"/>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>byjspark@schmc.ac.kr</t>
+        </is>
+      </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>https://www.schmc.ac.kr/bucheon/doctr/home.do?key=2947&amp;doctrNo=3540</t>
@@ -1024,7 +1036,11 @@
           <t>Principal Investigators</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n"/>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>heartonbrainmd@yuhs.ac</t>
+        </is>
+      </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
           <t>https://sev.severance.healthcare/sev/doctor/doctor-view.do?empNo=eXVoczIwMjBAKUApMuAmi0U3EuFuVaDODBFIMQ1O86v%2B%2FKVXhsSvUma5xMc%3D</t>

</xml_diff>